<commit_message>
oprava chyb reporty, index
</commit_message>
<xml_diff>
--- a/google_data/Pobočky/Prosek/Report Prosek.xlsx
+++ b/google_data/Pobočky/Prosek/Report Prosek.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1941" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1952" uniqueCount="716">
   <si>
     <t>Datum</t>
   </si>
@@ -1842,12 +1842,36 @@
     <t>Počet hodin</t>
   </si>
   <si>
+    <t>Šebesta Tomáš</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
     <t>Výdaje</t>
   </si>
   <si>
+    <t>Nováková Adéla</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>00:00</t>
+  </si>
+  <si>
     <t>Benzín</t>
   </si>
   <si>
+    <t>Fáberová Kateřina</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
     <t>Auta</t>
   </si>
   <si>
@@ -1941,16 +1965,13 @@
     <t>112:00</t>
   </si>
   <si>
-    <t>Šebesta Tomáš</t>
-  </si>
-  <si>
-    <t>95:30</t>
+    <t>123:00</t>
   </si>
   <si>
     <t>23:00</t>
   </si>
   <si>
-    <t>Nováková Adéla</t>
+    <t>104:00</t>
   </si>
   <si>
     <t>13:00</t>
@@ -1959,19 +1980,16 @@
     <t>Putna Jaroslav</t>
   </si>
   <si>
-    <t>117:00</t>
-  </si>
-  <si>
-    <t>Fáberová Kateřina</t>
-  </si>
-  <si>
-    <t>16:00</t>
+    <t>146:30</t>
+  </si>
+  <si>
+    <t>24:00</t>
   </si>
   <si>
     <t>7:00</t>
   </si>
   <si>
-    <t>12 min 35 s</t>
+    <t>12 min 31 s</t>
   </si>
   <si>
     <t>Manažeři</t>
@@ -13250,7 +13268,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="9">
-        <v>46191.0</v>
+        <v>46194.0</v>
       </c>
       <c r="E1" s="10"/>
       <c r="F1" s="11" t="s">
@@ -13299,7 +13317,7 @@
       <c r="A3" s="24"/>
       <c r="B3" s="25" t="str">
         <f>CHOOSE(WEEKDAY(D1), "Neděle", "Pondělí", "Úterý", "Středa", "Čtvrtek", "Pátek", "Sobota")</f>
-        <v>Čtvrtek</v>
+        <v>Neděle</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -13458,7 +13476,9 @@
       <c r="F11" s="44" t="s">
         <v>606</v>
       </c>
-      <c r="G11" s="45"/>
+      <c r="G11" s="45" t="s">
+        <v>607</v>
+      </c>
       <c r="I11" s="20"/>
       <c r="J11" s="46">
         <f>M2+M3+M4+M5+M6+M13+M14+M15+M16+M17+M9+M10+M11-I2</f>
@@ -13475,20 +13495,26 @@
         <f t="array" ref="A12">IF(ISBLANK(B12), 0, IF(ISNUMBER(MATCH(B12, HR!A:A, 0)), 0, IF(ISNUMBER(MATCH(B12, HR!B:B, 0)), INDEX(HR!V:V, MATCH(B12, HR!B:B, 0)) * (F12 * 24), 0)))</f>
         <v>0</v>
       </c>
-      <c r="B12" s="50"/>
-      <c r="C12" s="51"/>
-      <c r="D12" s="51"/>
+      <c r="B12" s="50" t="s">
+        <v>607</v>
+      </c>
+      <c r="C12" s="51" t="s">
+        <v>608</v>
+      </c>
+      <c r="D12" s="51" t="s">
+        <v>609</v>
+      </c>
       <c r="E12" s="52"/>
       <c r="F12" s="53" t="str">
         <f t="shared" ref="F12:F21" si="1">IF(OR(ISBLANK(B12), ISBLANK(D12), D12=0), "0:00", TEXT((IF(AND(TIMEVALUE(IF(ISBLANK(D12), "00:00", D12))&gt;=TIMEVALUE("00:00"), TIMEVALUE(IF(ISBLANK(D12), "00:00", D12))&lt;=TIMEVALUE("06:00")), TIMEVALUE(IF(ISBLANK(D12), "00:00", D12))+1, TIMEVALUE(IF(ISBLANK(D12), "00:00", D12))) - TIMEVALUE(IF(ISBLANK(C12), "00:00", C12)) - TIMEVALUE(IF(ISBLANK(E12), "00:00", E12))), "hh:mm"))
 </f>
-        <v>0:00</v>
+        <v>#VALUE!</v>
       </c>
       <c r="I12" s="20"/>
       <c r="J12" s="35"/>
       <c r="K12" s="20"/>
       <c r="L12" s="54" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="M12" s="18"/>
     </row>
@@ -13497,13 +13523,19 @@
         <f t="array" ref="A13">IF(ISBLANK(B13), 0, IF(ISNUMBER(MATCH(B13, HR!A:A, 0)), 0, IF(ISNUMBER(MATCH(B13, HR!B:B, 0)), INDEX(HR!V:V, MATCH(B13, HR!B:B, 0)) * (F13 * 24), 0)))</f>
         <v>0</v>
       </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
+      <c r="B13" s="50" t="s">
+        <v>611</v>
+      </c>
+      <c r="C13" s="51" t="s">
+        <v>612</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>613</v>
+      </c>
       <c r="E13" s="52"/>
       <c r="F13" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>0:00</v>
+        <v>07:00</v>
       </c>
       <c r="G13" s="27"/>
       <c r="H13" s="27"/>
@@ -13511,29 +13543,35 @@
       <c r="J13" s="35"/>
       <c r="K13" s="20"/>
       <c r="L13" s="22" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="M13" s="37"/>
     </row>
     <row r="14">
       <c r="A14" s="49">
         <f t="array" ref="A14">IF(ISBLANK(B14), 0, IF(ISNUMBER(MATCH(B14, HR!A:A, 0)), 0, IF(ISNUMBER(MATCH(B14, HR!B:B, 0)), INDEX(HR!V:V, MATCH(B14, HR!B:B, 0)) * (F14 * 24), 0)))</f>
-        <v>0</v>
-      </c>
-      <c r="B14" s="50"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
+        <v>1501.236</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>615</v>
+      </c>
+      <c r="C14" s="51" t="s">
+        <v>616</v>
+      </c>
+      <c r="D14" s="51" t="s">
+        <v>613</v>
+      </c>
       <c r="E14" s="55"/>
       <c r="F14" s="53" t="str">
         <f t="shared" si="1"/>
-        <v>0:00</v>
+        <v>06:00</v>
       </c>
       <c r="G14" s="56"/>
       <c r="I14" s="20"/>
       <c r="J14" s="35"/>
       <c r="K14" s="20"/>
       <c r="L14" s="57" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="M14" s="37"/>
     </row>
@@ -13554,7 +13592,7 @@
       <c r="J15" s="35"/>
       <c r="K15" s="20"/>
       <c r="L15" s="57" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="M15" s="37"/>
     </row>
@@ -13575,7 +13613,7 @@
       <c r="J16" s="35"/>
       <c r="K16" s="20"/>
       <c r="L16" s="57" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="M16" s="37"/>
     </row>
@@ -13598,7 +13636,7 @@
       <c r="J17" s="17"/>
       <c r="K17" s="18"/>
       <c r="L17" s="59" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
       <c r="M17" s="60">
         <f>sum(I25:I31)</f>
@@ -13619,7 +13657,7 @@
         <v>0:00</v>
       </c>
       <c r="G18" s="54" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="H18" s="27"/>
       <c r="I18" s="18"/>
@@ -13639,7 +13677,9 @@
         <f t="shared" si="1"/>
         <v>0:00</v>
       </c>
-      <c r="G19" s="45"/>
+      <c r="G19" s="45" t="s">
+        <v>611</v>
+      </c>
       <c r="I19" s="20"/>
       <c r="M19" s="62"/>
     </row>
@@ -13688,16 +13728,16 @@
       <c r="H22" s="27"/>
       <c r="I22" s="18"/>
       <c r="J22" s="70" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="K22" s="70" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="L22" s="71" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="M22" s="71" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
     </row>
     <row r="23">
@@ -13741,25 +13781,25 @@
         <v>606</v>
       </c>
       <c r="G24" s="75" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="H24" s="75" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="I24" s="76" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="J24" s="77" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="K24" s="78" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="L24" s="77" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
       <c r="M24" s="78" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
     </row>
     <row r="25">
@@ -13858,14 +13898,14 @@
         <v>0</v>
       </c>
       <c r="J27" s="89" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="K27" s="90"/>
       <c r="L27" s="77" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="M27" s="78" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
@@ -13962,10 +14002,10 @@
       <c r="J30" s="96"/>
       <c r="K30" s="96"/>
       <c r="L30" s="78" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="M30" s="78" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
     </row>
     <row r="31">
@@ -14003,7 +14043,7 @@
         <v>17</v>
       </c>
       <c r="C32" s="99" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
@@ -14086,11 +14126,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B12:B21">
-      <formula1>"Nedbal Michal,Ahurieva Viktoriia,Pešová Hana,Šebesta Tomáš,Coufal Jakub,Nováková Adéla,Makula Radek,Yarushynskyi Vladyslav,Gorol Patrik,Putna Jaroslav,Kopic Jakub,Fáberová Kateřina"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B25:B31">
       <formula1>"Hanibal Filip,Mikuš Pavel,Šmídová Sabina,Kormash Liubov,Vychivskyi Volodymyr,Hřebík Martin,Reischl Jan,Kulinič Michail,Kačena Stanislav"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="B12:B21">
+      <formula1>"Nedbal Michal,Pešová Hana,Šebesta Tomáš,Coufal Jakub,Nováková Adéla,Makula Radek,Yarushynskyi Vladyslav,Gorol Patrik,Putna Jaroslav,Kopic Jakub,Fáberová Kateřina"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="G11 G19">
+      <formula1>"Šebesta Tomáš,Nováková Adéla,Fáberová Kateřina"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -14124,7 +14167,7 @@
         <v>46174.0</v>
       </c>
       <c r="D1" s="108" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
       <c r="E1" s="109">
         <v>46203.0</v>
@@ -14152,18 +14195,18 @@
       <c r="D2" s="16"/>
       <c r="E2" s="18"/>
       <c r="F2" s="112">
-        <v>0.3180380822647522</v>
+        <v>0.31312068182483815</v>
       </c>
       <c r="H2" s="20"/>
       <c r="I2" s="113">
-        <v>575843.4400000001</v>
+        <v>693189.9400000001</v>
       </c>
       <c r="K2" s="20"/>
       <c r="L2" s="114" t="s">
         <v>589</v>
       </c>
       <c r="M2" s="115">
-        <v>238081.89000000007</v>
+        <v>290469.6900000001</v>
       </c>
       <c r="N2" s="116"/>
     </row>
@@ -14185,7 +14228,7 @@
         <v>590</v>
       </c>
       <c r="M3" s="120">
-        <v>90909.0</v>
+        <v>108075.0</v>
       </c>
       <c r="N3" s="116"/>
     </row>
@@ -14205,20 +14248,20 @@
         <v>591</v>
       </c>
       <c r="M4" s="120">
-        <v>98299.65</v>
+        <v>113157.65</v>
       </c>
       <c r="N4" s="116"/>
     </row>
     <row r="5">
       <c r="A5" s="121"/>
       <c r="B5" s="122" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
       <c r="E5" s="10"/>
       <c r="F5" s="123" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
@@ -14229,7 +14272,7 @@
         <v>593</v>
       </c>
       <c r="M5" s="120">
-        <v>73263.0</v>
+        <v>86888.1</v>
       </c>
       <c r="N5" s="116"/>
     </row>
@@ -14249,7 +14292,7 @@
         <v>594</v>
       </c>
       <c r="M6" s="120">
-        <v>4961.0</v>
+        <v>7858.6</v>
       </c>
       <c r="N6" s="116"/>
     </row>
@@ -14257,7 +14300,7 @@
       <c r="A7" s="125"/>
       <c r="B7" s="126">
         <f>TEXT(SUMPRODUCT((IFERROR(LEFT(D10:D30, FIND(":", D10:D30) - 1) * 60, 0) + IFERROR(MID(D10:D30, FIND(":", D10:D30) + 1, LEN(D10:D30) - FIND(":", D10:D30)), 0))), "[h]:mm")/60</f>
-        <v>336</v>
+        <v>409.5</v>
       </c>
       <c r="C7" s="27"/>
       <c r="D7" s="27"/>
@@ -14309,7 +14352,7 @@
         <v>602</v>
       </c>
       <c r="C9" s="138" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="D9" s="138" t="s">
         <v>606</v>
@@ -14319,48 +14362,48 @@
         <v>602</v>
       </c>
       <c r="G9" s="138" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="H9" s="138" t="s">
         <v>606</v>
       </c>
       <c r="I9" s="140" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="J9" s="141">
-        <v>7.100000000064028</v>
+        <v>7.100000000085856</v>
       </c>
       <c r="K9" s="10"/>
       <c r="L9" s="142" t="s">
         <v>597</v>
       </c>
       <c r="M9" s="120">
-        <v>42625.0</v>
+        <v>53801.0</v>
       </c>
       <c r="N9" s="116"/>
     </row>
     <row r="10" ht="18.75" customHeight="1">
       <c r="A10" s="143"/>
       <c r="B10" s="144" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="C10" s="145">
         <v>1.0</v>
       </c>
       <c r="D10" s="145" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
       <c r="E10" s="146" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="F10" s="144" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="G10" s="145">
         <v>10.0</v>
       </c>
       <c r="H10" s="145" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="I10" s="147">
         <v>49.0</v>
@@ -14378,16 +14421,16 @@
     <row r="11" ht="18.75" customHeight="1">
       <c r="A11" s="143"/>
       <c r="B11" s="144" t="s">
-        <v>640</v>
+        <v>607</v>
       </c>
       <c r="C11" s="145">
-        <v>11.0</v>
+        <v>14.0</v>
       </c>
       <c r="D11" s="145" t="s">
-        <v>641</v>
+        <v>648</v>
       </c>
       <c r="E11" s="146" t="s">
-        <v>642</v>
+        <v>649</v>
       </c>
       <c r="F11" s="144"/>
       <c r="G11" s="145"/>
@@ -14399,23 +14442,23 @@
         <v>596</v>
       </c>
       <c r="M11" s="149">
-        <v>21256.0</v>
+        <v>24603.0</v>
       </c>
       <c r="N11" s="116"/>
     </row>
     <row r="12" ht="18.75" customHeight="1">
       <c r="A12" s="143"/>
       <c r="B12" s="144" t="s">
-        <v>643</v>
+        <v>611</v>
       </c>
       <c r="C12" s="145">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
       <c r="D12" s="145" t="s">
-        <v>641</v>
+        <v>650</v>
       </c>
       <c r="E12" s="146" t="s">
-        <v>644</v>
+        <v>651</v>
       </c>
       <c r="F12" s="144"/>
       <c r="G12" s="145"/>
@@ -14424,7 +14467,7 @@
       <c r="J12" s="35"/>
       <c r="K12" s="20"/>
       <c r="L12" s="150" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="M12" s="18"/>
       <c r="N12" s="111"/>
@@ -14432,16 +14475,16 @@
     <row r="13" ht="18.75" customHeight="1">
       <c r="A13" s="143"/>
       <c r="B13" s="144" t="s">
-        <v>645</v>
+        <v>652</v>
       </c>
       <c r="C13" s="145">
-        <v>12.0</v>
+        <v>15.0</v>
       </c>
       <c r="D13" s="145" t="s">
-        <v>646</v>
+        <v>653</v>
       </c>
       <c r="E13" s="146" t="s">
-        <v>644</v>
+        <v>651</v>
       </c>
       <c r="F13" s="144"/>
       <c r="G13" s="145"/>
@@ -14450,26 +14493,26 @@
       <c r="J13" s="35"/>
       <c r="K13" s="20"/>
       <c r="L13" s="142" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="M13" s="120">
-        <v>1700.0</v>
+        <v>2400.0</v>
       </c>
       <c r="N13" s="116"/>
     </row>
     <row r="14" ht="18.75" customHeight="1">
       <c r="A14" s="143"/>
       <c r="B14" s="144" t="s">
-        <v>647</v>
+        <v>615</v>
       </c>
       <c r="C14" s="145">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="D14" s="145" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="E14" s="146" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="F14" s="144"/>
       <c r="G14" s="145"/>
@@ -14478,7 +14521,7 @@
       <c r="J14" s="35"/>
       <c r="K14" s="20"/>
       <c r="L14" s="151" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="M14" s="120">
         <v>0.0</v>
@@ -14491,7 +14534,7 @@
       <c r="C15" s="145"/>
       <c r="D15" s="145"/>
       <c r="E15" s="146" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="F15" s="144"/>
       <c r="G15" s="145"/>
@@ -14500,7 +14543,7 @@
       <c r="J15" s="35"/>
       <c r="K15" s="20"/>
       <c r="L15" s="151" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="M15" s="120">
         <v>140.0</v>
@@ -14520,10 +14563,10 @@
       <c r="J16" s="35"/>
       <c r="K16" s="20"/>
       <c r="L16" s="151" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="M16" s="120">
-        <v>1165.0</v>
+        <v>2354.0</v>
       </c>
       <c r="N16" s="116"/>
     </row>
@@ -14540,7 +14583,7 @@
       <c r="J17" s="17"/>
       <c r="K17" s="18"/>
       <c r="L17" s="153" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
       <c r="M17" s="154">
         <v>2205.0</v>
@@ -14574,16 +14617,16 @@
       <c r="H19" s="145"/>
       <c r="I19" s="147"/>
       <c r="J19" s="157" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="K19" s="158" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="L19" s="159" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="M19" s="160" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="N19" s="161"/>
     </row>
@@ -14614,16 +14657,16 @@
       <c r="H21" s="145"/>
       <c r="I21" s="147"/>
       <c r="J21" s="164">
-        <v>13.0</v>
+        <v>18.0</v>
       </c>
       <c r="K21" s="165">
-        <v>5894.6</v>
+        <v>8044.400000000001</v>
       </c>
       <c r="L21" s="166">
-        <v>24.0</v>
+        <v>29.0</v>
       </c>
       <c r="M21" s="167" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="N21" s="156"/>
     </row>
@@ -14638,16 +14681,16 @@
       <c r="H22" s="145"/>
       <c r="I22" s="147"/>
       <c r="J22" s="168" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="K22" s="169" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="L22" s="170" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
       <c r="M22" s="171" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="N22" s="156"/>
     </row>
@@ -14681,13 +14724,13 @@
         <v>9.0</v>
       </c>
       <c r="K24" s="166">
-        <v>1461.0</v>
+        <v>1783.0</v>
       </c>
       <c r="L24" s="166">
-        <v>140.0</v>
+        <v>175.0</v>
       </c>
       <c r="M24" s="173">
-        <v>28.0</v>
+        <v>34.0</v>
       </c>
       <c r="N24" s="156"/>
     </row>
@@ -14702,14 +14745,14 @@
       <c r="H25" s="145"/>
       <c r="I25" s="147"/>
       <c r="J25" s="174" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="K25" s="90"/>
       <c r="L25" s="175" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="M25" s="176" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="N25" s="156"/>
     </row>
@@ -14740,14 +14783,14 @@
       <c r="H27" s="145"/>
       <c r="I27" s="147"/>
       <c r="J27" s="178">
-        <v>12.0</v>
+        <v>15.0</v>
       </c>
       <c r="K27" s="94"/>
       <c r="L27" s="179">
-        <v>0.14754623440285208</v>
+        <v>0.14638171426097124</v>
       </c>
       <c r="M27" s="180">
-        <v>19.0</v>
+        <v>24.0</v>
       </c>
       <c r="N27" s="156"/>
     </row>
@@ -14763,10 +14806,10 @@
       <c r="I28" s="147"/>
       <c r="J28" s="181"/>
       <c r="L28" s="182" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="M28" s="176" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="N28" s="156"/>
     </row>
@@ -14798,10 +14841,10 @@
       <c r="J30" s="17"/>
       <c r="K30" s="27"/>
       <c r="L30" s="183">
-        <v>0.852453765597148</v>
+        <v>0.8536182857390289</v>
       </c>
       <c r="M30" s="184">
-        <v>0.11956420825906121</v>
+        <v>0.12281790277146315</v>
       </c>
       <c r="N30" s="156"/>
     </row>
@@ -15151,7 +15194,7 @@
       <c r="B9" s="4"/>
       <c r="C9" s="186"/>
       <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="E9" s="185"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -15185,7 +15228,7 @@
       <c r="B10" s="4"/>
       <c r="C10" s="186"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="E10" s="185"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -15395,7 +15438,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="K16" s="185"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
@@ -15457,13 +15500,13 @@
       <c r="B18" s="186"/>
       <c r="C18" s="186"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="185"/>
+      <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
-      <c r="K18" s="185"/>
+      <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
@@ -15491,7 +15534,7 @@
       <c r="B19" s="4"/>
       <c r="C19" s="186"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="185"/>
+      <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -15593,7 +15636,7 @@
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="185"/>
+      <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -15695,7 +15738,7 @@
       <c r="B25" s="186"/>
       <c r="C25" s="186"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="185"/>
+      <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -15729,7 +15772,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="186"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="185"/>
+      <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -15802,7 +15845,7 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
+      <c r="K28" s="185"/>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
@@ -15830,13 +15873,13 @@
       <c r="B29" s="186"/>
       <c r="C29" s="186"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="185"/>
+      <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
-      <c r="K29" s="185"/>
+      <c r="K29" s="4"/>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
@@ -15864,7 +15907,7 @@
       <c r="B30" s="186"/>
       <c r="C30" s="186"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="185"/>
+      <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -15898,7 +15941,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="186"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="185"/>
+      <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -15966,13 +16009,13 @@
       <c r="B33" s="4"/>
       <c r="C33" s="186"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="E33" s="185"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
+      <c r="K33" s="185"/>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
@@ -16006,7 +16049,7 @@
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
-      <c r="K34" s="185"/>
+      <c r="K34" s="4"/>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
@@ -16068,7 +16111,7 @@
       <c r="B36" s="4"/>
       <c r="C36" s="186"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="E36" s="185"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -16102,7 +16145,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="186"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="185"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -16136,7 +16179,7 @@
       <c r="B38" s="186"/>
       <c r="C38" s="186"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="185"/>
+      <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -16170,7 +16213,7 @@
       <c r="B39" s="4"/>
       <c r="C39" s="186"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="E39" s="185"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -16210,7 +16253,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="185"/>
+      <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
@@ -16272,7 +16315,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="186"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="E42" s="185"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -16312,7 +16355,7 @@
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
+      <c r="K43" s="185"/>
       <c r="L43" s="4"/>
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
@@ -16408,7 +16451,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="186"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="185"/>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -16448,7 +16491,7 @@
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
       <c r="J47" s="4"/>
-      <c r="K47" s="185"/>
+      <c r="K47" s="4"/>
       <c r="L47" s="4"/>
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
@@ -16476,13 +16519,13 @@
       <c r="B48" s="4"/>
       <c r="C48" s="186"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="E48" s="185"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
+      <c r="K48" s="185"/>
       <c r="L48" s="4"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
@@ -16510,7 +16553,7 @@
       <c r="B49" s="4"/>
       <c r="C49" s="186"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="E49" s="185"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -16544,7 +16587,7 @@
       <c r="B50" s="4"/>
       <c r="C50" s="186"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="185"/>
+      <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -16578,7 +16621,7 @@
       <c r="B51" s="4"/>
       <c r="C51" s="186"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="E51" s="185"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -16646,7 +16689,7 @@
       <c r="B53" s="4"/>
       <c r="C53" s="186"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="185"/>
+      <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -16720,7 +16763,7 @@
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
-      <c r="K55" s="185"/>
+      <c r="K55" s="4"/>
       <c r="L55" s="4"/>
       <c r="M55" s="4"/>
       <c r="N55" s="4"/>
@@ -16748,13 +16791,13 @@
       <c r="B56" s="4"/>
       <c r="C56" s="186"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
+      <c r="E56" s="185"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
+      <c r="K56" s="185"/>
       <c r="L56" s="4"/>
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
@@ -16782,7 +16825,7 @@
       <c r="B57" s="4"/>
       <c r="C57" s="186"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="E57" s="185"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -16822,7 +16865,7 @@
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
-      <c r="K58" s="185"/>
+      <c r="K58" s="4"/>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
@@ -16884,7 +16927,7 @@
       <c r="B60" s="4"/>
       <c r="C60" s="186"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="185"/>
+      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -16986,7 +17029,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="186"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="E63" s="185"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -17054,7 +17097,7 @@
       <c r="B65" s="4"/>
       <c r="C65" s="186"/>
       <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
+      <c r="E65" s="185"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -17122,7 +17165,7 @@
       <c r="B67" s="4"/>
       <c r="C67" s="186"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="E67" s="185"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -17229,7 +17272,7 @@
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
       <c r="J70" s="4"/>
-      <c r="K70" s="185"/>
+      <c r="K70" s="4"/>
       <c r="L70" s="4"/>
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
@@ -17257,7 +17300,7 @@
       <c r="B71" s="4"/>
       <c r="C71" s="186"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="185"/>
+      <c r="E71" s="4"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -17291,13 +17334,13 @@
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
-      <c r="E72" s="185"/>
+      <c r="E72" s="4"/>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
       <c r="J72" s="4"/>
-      <c r="K72" s="185"/>
+      <c r="K72" s="4"/>
       <c r="L72" s="4"/>
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
@@ -17325,13 +17368,13 @@
       <c r="B73" s="4"/>
       <c r="C73" s="186"/>
       <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
+      <c r="E73" s="185"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
       <c r="J73" s="4"/>
-      <c r="K73" s="4"/>
+      <c r="K73" s="185"/>
       <c r="L73" s="4"/>
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
@@ -17359,7 +17402,7 @@
       <c r="B74" s="186"/>
       <c r="C74" s="186"/>
       <c r="D74" s="4"/>
-      <c r="E74" s="4"/>
+      <c r="E74" s="185"/>
       <c r="F74" s="4"/>
       <c r="G74" s="4"/>
       <c r="H74" s="4"/>
@@ -17427,7 +17470,7 @@
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
-      <c r="E76" s="185"/>
+      <c r="E76" s="4"/>
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
@@ -17495,7 +17538,7 @@
       <c r="B78" s="4"/>
       <c r="C78" s="186"/>
       <c r="D78" s="4"/>
-      <c r="E78" s="185"/>
+      <c r="E78" s="4"/>
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
@@ -17535,7 +17578,7 @@
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
       <c r="J79" s="4"/>
-      <c r="K79" s="4"/>
+      <c r="K79" s="185"/>
       <c r="L79" s="4"/>
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
@@ -17569,7 +17612,7 @@
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
       <c r="J80" s="4"/>
-      <c r="K80" s="185"/>
+      <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
@@ -17637,7 +17680,7 @@
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
       <c r="J82" s="4"/>
-      <c r="K82" s="4"/>
+      <c r="K82" s="185"/>
       <c r="L82" s="4"/>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
@@ -17665,7 +17708,7 @@
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
-      <c r="E83" s="185"/>
+      <c r="E83" s="4"/>
       <c r="F83" s="4"/>
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
@@ -17699,7 +17742,7 @@
       <c r="B84" s="4"/>
       <c r="C84" s="186"/>
       <c r="D84" s="4"/>
-      <c r="E84" s="185"/>
+      <c r="E84" s="4"/>
       <c r="F84" s="4"/>
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
@@ -17773,7 +17816,7 @@
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
-      <c r="K86" s="4"/>
+      <c r="K86" s="185"/>
       <c r="L86" s="4"/>
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
@@ -17835,7 +17878,7 @@
       <c r="B88" s="4"/>
       <c r="C88" s="186"/>
       <c r="D88" s="4"/>
-      <c r="E88" s="185"/>
+      <c r="E88" s="4"/>
       <c r="F88" s="4"/>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
@@ -17875,7 +17918,7 @@
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
       <c r="J89" s="4"/>
-      <c r="K89" s="4"/>
+      <c r="K89" s="185"/>
       <c r="L89" s="4"/>
       <c r="M89" s="4"/>
       <c r="N89" s="4"/>
@@ -17903,7 +17946,7 @@
       <c r="B90" s="4"/>
       <c r="C90" s="186"/>
       <c r="D90" s="4"/>
-      <c r="E90" s="185"/>
+      <c r="E90" s="4"/>
       <c r="F90" s="4"/>
       <c r="G90" s="4"/>
       <c r="H90" s="4"/>
@@ -17969,7 +18012,7 @@
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
       <c r="D92" s="4"/>
-      <c r="E92" s="185"/>
+      <c r="E92" s="4"/>
       <c r="F92" s="4"/>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
@@ -18006,12 +18049,12 @@
       <c r="F93" s="4"/>
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
-      <c r="I93" s="185"/>
-      <c r="J93" s="185"/>
+      <c r="I93" s="4"/>
+      <c r="J93" s="4"/>
       <c r="K93" s="185"/>
       <c r="L93" s="4"/>
       <c r="M93" s="4"/>
-      <c r="N93" s="185"/>
+      <c r="N93" s="4"/>
       <c r="O93" s="4"/>
       <c r="P93" s="4"/>
       <c r="Q93" s="185"/>
@@ -18036,7 +18079,7 @@
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
       <c r="D94" s="4"/>
-      <c r="E94" s="185"/>
+      <c r="E94" s="4"/>
       <c r="F94" s="4"/>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
@@ -18069,16 +18112,16 @@
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
       <c r="D95" s="4"/>
-      <c r="E95" s="185"/>
+      <c r="E95" s="4"/>
       <c r="F95" s="4"/>
       <c r="G95" s="4"/>
       <c r="H95" s="4"/>
-      <c r="I95" s="185"/>
-      <c r="J95" s="185"/>
+      <c r="I95" s="4"/>
+      <c r="J95" s="4"/>
       <c r="K95" s="185"/>
       <c r="L95" s="4"/>
       <c r="M95" s="4"/>
-      <c r="N95" s="185"/>
+      <c r="N95" s="4"/>
       <c r="O95" s="4"/>
       <c r="P95" s="4"/>
       <c r="Q95" s="185"/>
@@ -18102,7 +18145,7 @@
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
       <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
+      <c r="E96" s="185"/>
       <c r="F96" s="4"/>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
@@ -18135,7 +18178,7 @@
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
       <c r="D97" s="4"/>
-      <c r="E97" s="185"/>
+      <c r="E97" s="4"/>
       <c r="F97" s="4"/>
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
@@ -18169,7 +18212,7 @@
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
       <c r="D98" s="4"/>
-      <c r="E98" s="185"/>
+      <c r="E98" s="4"/>
       <c r="F98" s="4"/>
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
@@ -18198,22 +18241,22 @@
       <c r="AF98" s="185"/>
     </row>
     <row r="99">
-      <c r="A99" s="185"/>
-      <c r="B99" s="185"/>
-      <c r="C99" s="187"/>
-      <c r="D99" s="185"/>
-      <c r="E99" s="185"/>
-      <c r="F99" s="185"/>
-      <c r="G99" s="185"/>
-      <c r="H99" s="185"/>
-      <c r="I99" s="185"/>
-      <c r="J99" s="185"/>
+      <c r="A99" s="4"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="186"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="4"/>
+      <c r="H99" s="4"/>
+      <c r="I99" s="4"/>
+      <c r="J99" s="4"/>
       <c r="K99" s="185"/>
-      <c r="L99" s="185"/>
-      <c r="M99" s="185"/>
-      <c r="N99" s="185"/>
-      <c r="O99" s="185"/>
-      <c r="P99" s="185"/>
+      <c r="L99" s="4"/>
+      <c r="M99" s="4"/>
+      <c r="N99" s="4"/>
+      <c r="O99" s="4"/>
+      <c r="P99" s="4"/>
       <c r="Q99" s="185"/>
       <c r="R99" s="185"/>
       <c r="S99" s="185"/>
@@ -18232,22 +18275,22 @@
       <c r="AF99" s="185"/>
     </row>
     <row r="100">
-      <c r="A100" s="185"/>
-      <c r="B100" s="185"/>
-      <c r="C100" s="187"/>
-      <c r="D100" s="185"/>
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="186"/>
+      <c r="D100" s="4"/>
       <c r="E100" s="185"/>
-      <c r="F100" s="185"/>
-      <c r="G100" s="185"/>
-      <c r="H100" s="185"/>
-      <c r="I100" s="185"/>
-      <c r="J100" s="185"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="4"/>
+      <c r="J100" s="4"/>
       <c r="K100" s="185"/>
-      <c r="L100" s="185"/>
-      <c r="M100" s="185"/>
-      <c r="N100" s="185"/>
-      <c r="O100" s="185"/>
-      <c r="P100" s="185"/>
+      <c r="L100" s="4"/>
+      <c r="M100" s="4"/>
+      <c r="N100" s="4"/>
+      <c r="O100" s="4"/>
+      <c r="P100" s="4"/>
       <c r="Q100" s="185"/>
       <c r="R100" s="185"/>
       <c r="S100" s="185"/>
@@ -18265,22 +18308,22 @@
       <c r="AF100" s="185"/>
     </row>
     <row r="101">
-      <c r="A101" s="185"/>
-      <c r="B101" s="185"/>
-      <c r="C101" s="185"/>
-      <c r="D101" s="185"/>
+      <c r="A101" s="4"/>
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
       <c r="E101" s="185"/>
-      <c r="F101" s="185"/>
-      <c r="G101" s="185"/>
-      <c r="H101" s="185"/>
-      <c r="I101" s="185"/>
-      <c r="J101" s="185"/>
+      <c r="F101" s="4"/>
+      <c r="G101" s="4"/>
+      <c r="H101" s="4"/>
+      <c r="I101" s="4"/>
+      <c r="J101" s="4"/>
       <c r="K101" s="185"/>
-      <c r="L101" s="185"/>
-      <c r="M101" s="185"/>
-      <c r="N101" s="185"/>
-      <c r="O101" s="185"/>
-      <c r="P101" s="185"/>
+      <c r="L101" s="4"/>
+      <c r="M101" s="4"/>
+      <c r="N101" s="4"/>
+      <c r="O101" s="4"/>
+      <c r="P101" s="4"/>
       <c r="Q101" s="185"/>
       <c r="R101" s="185"/>
       <c r="S101" s="185"/>
@@ -18298,22 +18341,22 @@
       <c r="AF101" s="185"/>
     </row>
     <row r="102">
-      <c r="A102" s="185"/>
-      <c r="B102" s="185"/>
-      <c r="C102" s="187"/>
-      <c r="D102" s="185"/>
+      <c r="A102" s="4"/>
+      <c r="B102" s="4"/>
+      <c r="C102" s="186"/>
+      <c r="D102" s="4"/>
       <c r="E102" s="185"/>
-      <c r="F102" s="185"/>
-      <c r="G102" s="185"/>
-      <c r="H102" s="185"/>
-      <c r="I102" s="185"/>
-      <c r="J102" s="185"/>
+      <c r="F102" s="4"/>
+      <c r="G102" s="4"/>
+      <c r="H102" s="4"/>
+      <c r="I102" s="4"/>
+      <c r="J102" s="4"/>
       <c r="K102" s="185"/>
-      <c r="L102" s="185"/>
-      <c r="M102" s="185"/>
-      <c r="N102" s="185"/>
-      <c r="O102" s="185"/>
-      <c r="P102" s="185"/>
+      <c r="L102" s="4"/>
+      <c r="M102" s="4"/>
+      <c r="N102" s="4"/>
+      <c r="O102" s="4"/>
+      <c r="P102" s="4"/>
       <c r="Q102" s="185"/>
       <c r="R102" s="185"/>
       <c r="S102" s="185"/>
@@ -18331,22 +18374,22 @@
       <c r="AF102" s="185"/>
     </row>
     <row r="103">
-      <c r="A103" s="185"/>
-      <c r="B103" s="185"/>
-      <c r="C103" s="187"/>
-      <c r="D103" s="185"/>
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
+      <c r="C103" s="186"/>
+      <c r="D103" s="4"/>
       <c r="E103" s="185"/>
-      <c r="F103" s="185"/>
-      <c r="G103" s="185"/>
-      <c r="H103" s="185"/>
-      <c r="I103" s="185"/>
-      <c r="J103" s="185"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="4"/>
+      <c r="H103" s="4"/>
+      <c r="I103" s="4"/>
+      <c r="J103" s="4"/>
       <c r="K103" s="185"/>
-      <c r="L103" s="185"/>
-      <c r="M103" s="185"/>
-      <c r="N103" s="185"/>
-      <c r="O103" s="185"/>
-      <c r="P103" s="185"/>
+      <c r="L103" s="4"/>
+      <c r="M103" s="4"/>
+      <c r="N103" s="4"/>
+      <c r="O103" s="4"/>
+      <c r="P103" s="4"/>
       <c r="Q103" s="185"/>
       <c r="R103" s="185"/>
       <c r="S103" s="185"/>
@@ -18365,22 +18408,22 @@
       <c r="AF103" s="185"/>
     </row>
     <row r="104">
-      <c r="A104" s="185"/>
-      <c r="B104" s="185"/>
-      <c r="C104" s="185"/>
-      <c r="D104" s="185"/>
-      <c r="E104" s="185"/>
-      <c r="F104" s="185"/>
-      <c r="G104" s="185"/>
-      <c r="H104" s="185"/>
-      <c r="I104" s="185"/>
-      <c r="J104" s="185"/>
+      <c r="A104" s="4"/>
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
+      <c r="G104" s="4"/>
+      <c r="H104" s="4"/>
+      <c r="I104" s="4"/>
+      <c r="J104" s="4"/>
       <c r="K104" s="185"/>
-      <c r="L104" s="185"/>
-      <c r="M104" s="185"/>
-      <c r="N104" s="185"/>
-      <c r="O104" s="185"/>
-      <c r="P104" s="185"/>
+      <c r="L104" s="4"/>
+      <c r="M104" s="4"/>
+      <c r="N104" s="4"/>
+      <c r="O104" s="4"/>
+      <c r="P104" s="4"/>
       <c r="Q104" s="185"/>
       <c r="R104" s="185"/>
       <c r="S104" s="185"/>
@@ -18399,22 +18442,22 @@
       <c r="AF104" s="185"/>
     </row>
     <row r="105">
-      <c r="A105" s="185"/>
-      <c r="B105" s="185"/>
-      <c r="C105" s="187"/>
-      <c r="D105" s="185"/>
-      <c r="E105" s="185"/>
-      <c r="F105" s="185"/>
-      <c r="G105" s="185"/>
-      <c r="H105" s="185"/>
-      <c r="I105" s="185"/>
-      <c r="J105" s="185"/>
+      <c r="A105" s="4"/>
+      <c r="B105" s="4"/>
+      <c r="C105" s="186"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="4"/>
+      <c r="H105" s="4"/>
+      <c r="I105" s="4"/>
+      <c r="J105" s="4"/>
       <c r="K105" s="185"/>
-      <c r="L105" s="185"/>
-      <c r="M105" s="185"/>
-      <c r="N105" s="185"/>
-      <c r="O105" s="185"/>
-      <c r="P105" s="185"/>
+      <c r="L105" s="4"/>
+      <c r="M105" s="4"/>
+      <c r="N105" s="4"/>
+      <c r="O105" s="4"/>
+      <c r="P105" s="4"/>
       <c r="Q105" s="185"/>
       <c r="R105" s="185"/>
       <c r="S105" s="185"/>
@@ -18433,22 +18476,22 @@
       <c r="AF105" s="185"/>
     </row>
     <row r="106">
-      <c r="A106" s="185"/>
-      <c r="B106" s="185"/>
-      <c r="C106" s="185"/>
-      <c r="D106" s="185"/>
+      <c r="A106" s="4"/>
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="4"/>
       <c r="E106" s="185"/>
-      <c r="F106" s="185"/>
-      <c r="G106" s="185"/>
-      <c r="H106" s="185"/>
-      <c r="I106" s="185"/>
-      <c r="J106" s="185"/>
+      <c r="F106" s="4"/>
+      <c r="G106" s="4"/>
+      <c r="H106" s="4"/>
+      <c r="I106" s="4"/>
+      <c r="J106" s="4"/>
       <c r="K106" s="185"/>
-      <c r="L106" s="185"/>
-      <c r="M106" s="185"/>
-      <c r="N106" s="185"/>
-      <c r="O106" s="185"/>
-      <c r="P106" s="185"/>
+      <c r="L106" s="4"/>
+      <c r="M106" s="4"/>
+      <c r="N106" s="4"/>
+      <c r="O106" s="4"/>
+      <c r="P106" s="4"/>
       <c r="Q106" s="185"/>
       <c r="R106" s="185"/>
       <c r="S106" s="185"/>
@@ -18467,22 +18510,22 @@
       <c r="AF106" s="185"/>
     </row>
     <row r="107">
-      <c r="A107" s="185"/>
-      <c r="B107" s="185"/>
-      <c r="C107" s="185"/>
-      <c r="D107" s="185"/>
-      <c r="E107" s="185"/>
-      <c r="F107" s="185"/>
-      <c r="G107" s="185"/>
-      <c r="H107" s="185"/>
-      <c r="I107" s="185"/>
-      <c r="J107" s="185"/>
+      <c r="A107" s="4"/>
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="4"/>
       <c r="K107" s="185"/>
-      <c r="L107" s="185"/>
-      <c r="M107" s="185"/>
-      <c r="N107" s="185"/>
-      <c r="O107" s="185"/>
-      <c r="P107" s="185"/>
+      <c r="L107" s="4"/>
+      <c r="M107" s="4"/>
+      <c r="N107" s="4"/>
+      <c r="O107" s="4"/>
+      <c r="P107" s="4"/>
       <c r="Q107" s="185"/>
       <c r="R107" s="185"/>
       <c r="S107" s="185"/>
@@ -18501,22 +18544,22 @@
       <c r="AF107" s="185"/>
     </row>
     <row r="108">
-      <c r="A108" s="185"/>
-      <c r="B108" s="185"/>
-      <c r="C108" s="187"/>
-      <c r="D108" s="185"/>
+      <c r="A108" s="4"/>
+      <c r="B108" s="4"/>
+      <c r="C108" s="186"/>
+      <c r="D108" s="4"/>
       <c r="E108" s="185"/>
-      <c r="F108" s="185"/>
-      <c r="G108" s="185"/>
-      <c r="H108" s="185"/>
-      <c r="I108" s="185"/>
-      <c r="J108" s="185"/>
+      <c r="F108" s="4"/>
+      <c r="G108" s="4"/>
+      <c r="H108" s="4"/>
+      <c r="I108" s="4"/>
+      <c r="J108" s="4"/>
       <c r="K108" s="185"/>
-      <c r="L108" s="185"/>
-      <c r="M108" s="185"/>
-      <c r="N108" s="185"/>
-      <c r="O108" s="185"/>
-      <c r="P108" s="185"/>
+      <c r="L108" s="4"/>
+      <c r="M108" s="4"/>
+      <c r="N108" s="4"/>
+      <c r="O108" s="4"/>
+      <c r="P108" s="4"/>
       <c r="Q108" s="185"/>
       <c r="R108" s="185"/>
       <c r="S108" s="185"/>
@@ -18535,22 +18578,22 @@
       <c r="AF108" s="185"/>
     </row>
     <row r="109">
-      <c r="A109" s="185"/>
-      <c r="B109" s="185"/>
-      <c r="C109" s="185"/>
-      <c r="D109" s="185"/>
-      <c r="E109" s="185"/>
-      <c r="F109" s="185"/>
-      <c r="G109" s="185"/>
-      <c r="H109" s="185"/>
-      <c r="I109" s="185"/>
-      <c r="J109" s="185"/>
+      <c r="A109" s="4"/>
+      <c r="B109" s="4"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="4"/>
+      <c r="E109" s="4"/>
+      <c r="F109" s="4"/>
+      <c r="G109" s="4"/>
+      <c r="H109" s="4"/>
+      <c r="I109" s="4"/>
+      <c r="J109" s="4"/>
       <c r="K109" s="185"/>
-      <c r="L109" s="185"/>
-      <c r="M109" s="185"/>
-      <c r="N109" s="185"/>
-      <c r="O109" s="185"/>
-      <c r="P109" s="185"/>
+      <c r="L109" s="4"/>
+      <c r="M109" s="4"/>
+      <c r="N109" s="4"/>
+      <c r="O109" s="4"/>
+      <c r="P109" s="4"/>
       <c r="Q109" s="185"/>
       <c r="R109" s="185"/>
       <c r="S109" s="185"/>
@@ -19039,6 +19082,7 @@
       <c r="O124" s="185"/>
       <c r="P124" s="185"/>
       <c r="Q124" s="185"/>
+      <c r="R124" s="185"/>
       <c r="S124" s="185"/>
       <c r="T124" s="185"/>
       <c r="U124" s="185"/>
@@ -19047,10 +19091,42 @@
       <c r="X124" s="185"/>
       <c r="Y124" s="185"/>
       <c r="Z124" s="185"/>
+      <c r="AA124" s="185"/>
       <c r="AB124" s="185"/>
       <c r="AC124" s="185"/>
+      <c r="AD124" s="185"/>
       <c r="AE124" s="185"/>
       <c r="AF124" s="185"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="185"/>
+      <c r="B125" s="185"/>
+      <c r="C125" s="185"/>
+      <c r="D125" s="185"/>
+      <c r="E125" s="185"/>
+      <c r="F125" s="185"/>
+      <c r="G125" s="185"/>
+      <c r="H125" s="185"/>
+      <c r="I125" s="185"/>
+      <c r="J125" s="185"/>
+      <c r="K125" s="185"/>
+      <c r="L125" s="185"/>
+      <c r="M125" s="185"/>
+      <c r="O125" s="185"/>
+      <c r="P125" s="185"/>
+      <c r="Q125" s="185"/>
+      <c r="S125" s="185"/>
+      <c r="T125" s="185"/>
+      <c r="U125" s="185"/>
+      <c r="V125" s="185"/>
+      <c r="W125" s="185"/>
+      <c r="X125" s="185"/>
+      <c r="Y125" s="185"/>
+      <c r="Z125" s="185"/>
+      <c r="AB125" s="185"/>
+      <c r="AC125" s="185"/>
+      <c r="AE125" s="185"/>
+      <c r="AF125" s="185"/>
     </row>
     <row r="128">
       <c r="C128" s="187"/>
@@ -19226,10 +19302,10 @@
     </row>
     <row r="4">
       <c r="A4" s="191" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="B4" s="191" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="C4" s="2" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Manažer")</f>
@@ -19481,7 +19557,7 @@
       </c>
       <c r="B8" s="192" t="str">
         <f>IF(OR(E8=Report!$B$1, F8=Report!$B$1, G8=Report!$B$1, H8=Report!$B$1), D8, "")</f>
-        <v>Ahurieva Viktoriia</v>
+        <v/>
       </c>
       <c r="C8" s="2" t="b">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
@@ -19504,8 +19580,8 @@
         <v>Výroba</v>
       </c>
       <c r="H8" s="2" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Prosek")</f>
-        <v>Prosek</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zličín")</f>
+        <v>Zličín</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -19943,8 +20019,8 @@
         <v>Malešice</v>
       </c>
       <c r="F15" s="2" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zličín")</f>
-        <v>Zličín</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Bolevec")</f>
+        <v>Bolevec</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -61061,7 +61137,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="194" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -61093,28 +61169,28 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="I2" s="185"/>
       <c r="J2" s="185"/>
@@ -61143,22 +61219,22 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="C3" s="185"/>
       <c r="D3" s="185"/>
       <c r="E3" s="4" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="F3" s="185"/>
       <c r="G3" s="4" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="I3" s="185"/>
       <c r="J3" s="185"/>
@@ -61180,20 +61256,20 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="D4" s="185"/>
       <c r="E4" s="4" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G4" s="185"/>
       <c r="H4" s="185"/>
@@ -61217,18 +61293,18 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="B5" s="185"/>
       <c r="C5" s="4" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="E5" s="185"/>
       <c r="F5" s="4" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="G5" s="185"/>
       <c r="H5" s="185"/>
@@ -61255,15 +61331,15 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="C6" s="185"/>
       <c r="D6" s="4" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="E6" s="185"/>
       <c r="F6" s="4" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="G6" s="185"/>
       <c r="H6" s="185"/>
@@ -61290,14 +61366,14 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="C7" s="185"/>
       <c r="D7" s="4" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="G7" s="185"/>
       <c r="I7" s="185"/>
@@ -61321,14 +61397,14 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="F8" s="185"/>
       <c r="H8" s="4" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="I8" s="185"/>
       <c r="J8" s="185"/>
@@ -61353,17 +61429,17 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="D9" s="185"/>
       <c r="E9" s="4" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="H9" s="185"/>
       <c r="I9" s="185"/>
@@ -61388,14 +61464,14 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="F10" s="185"/>
       <c r="G10" s="4" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="I10" s="185"/>
       <c r="J10" s="185"/>
@@ -61608,7 +61684,7 @@
       <c r="Y19" s="185"/>
       <c r="Z19" s="185"/>
       <c r="AA19" s="4" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="AB19" s="4">
         <v>-11.0</v>
@@ -61933,7 +62009,7 @@
       <c r="Y30" s="185"/>
       <c r="Z30" s="185"/>
       <c r="AA30" s="4" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="AB30" s="4">
         <v>-8.0</v>
@@ -62054,7 +62130,7 @@
       <c r="Y34" s="185"/>
       <c r="Z34" s="185"/>
       <c r="AA34" s="4" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="AB34" s="4">
         <v>0.0</v>
@@ -62173,7 +62249,7 @@
       <c r="Y38" s="185"/>
       <c r="Z38" s="185"/>
       <c r="AA38" s="4" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="AB38" s="4">
         <v>-12.0</v>
@@ -62207,7 +62283,7 @@
       <c r="Y39" s="185"/>
       <c r="Z39" s="185"/>
       <c r="AA39" s="4" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="AB39" s="4">
         <v>0.0</v>
@@ -62299,7 +62375,7 @@
       <c r="Y42" s="185"/>
       <c r="Z42" s="185"/>
       <c r="AA42" s="4" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="AB42" s="4">
         <v>6.0</v>
@@ -62478,7 +62554,7 @@
       <c r="Y48" s="185"/>
       <c r="Z48" s="185"/>
       <c r="AA48" s="4" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="AB48" s="4">
         <v>-13.0</v>
@@ -62599,7 +62675,7 @@
       <c r="Y52" s="185"/>
       <c r="Z52" s="185"/>
       <c r="AA52" s="4" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="AB52" s="4">
         <v>5.0</v>
@@ -62807,7 +62883,7 @@
       <c r="Y59" s="185"/>
       <c r="Z59" s="185"/>
       <c r="AA59" s="4" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="AB59" s="4">
         <v>-9.0</v>
@@ -62928,7 +63004,7 @@
       <c r="Y63" s="185"/>
       <c r="Z63" s="185"/>
       <c r="AA63" s="4" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="AB63" s="4">
         <v>-19.0</v>
@@ -63136,7 +63212,7 @@
       <c r="Y70" s="185"/>
       <c r="Z70" s="185"/>
       <c r="AA70" s="4" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="AB70" s="4">
         <v>-14.0</v>
@@ -63605,7 +63681,7 @@
       <c r="Y86" s="185"/>
       <c r="Z86" s="185"/>
       <c r="AA86" s="4" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="AB86" s="4">
         <v>-21.0</v>
@@ -63639,7 +63715,7 @@
       <c r="Y87" s="185"/>
       <c r="Z87" s="185"/>
       <c r="AA87" s="4" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="AB87" s="4">
         <v>-7.0</v>
@@ -63673,7 +63749,7 @@
       <c r="Y88" s="185"/>
       <c r="Z88" s="185"/>
       <c r="AA88" s="4" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="AB88" s="4">
         <v>-10.0</v>
@@ -63707,7 +63783,7 @@
       <c r="Y89" s="185"/>
       <c r="Z89" s="185"/>
       <c r="AA89" s="4" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="AB89" s="4">
         <v>-6.0</v>
@@ -63800,7 +63876,7 @@
       <c r="Y92" s="185"/>
       <c r="Z92" s="185"/>
       <c r="AA92" s="4" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="AB92" s="4">
         <v>-17.0</v>
@@ -64066,7 +64142,7 @@
       <c r="Y101" s="185"/>
       <c r="Z101" s="185"/>
       <c r="AA101" s="4" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="AB101" s="4">
         <v>-6.0</v>
@@ -64100,7 +64176,7 @@
       <c r="Y102" s="185"/>
       <c r="Z102" s="185"/>
       <c r="AA102" s="4" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="AB102" s="4">
         <v>1.0</v>
@@ -64192,7 +64268,7 @@
       <c r="Y105" s="185"/>
       <c r="Z105" s="185"/>
       <c r="AA105" s="4" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="AB105" s="4">
         <v>-2.0</v>
@@ -64255,7 +64331,7 @@
       <c r="Y107" s="185"/>
       <c r="Z107" s="185"/>
       <c r="AA107" s="4" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="AB107" s="4">
         <v>-12.0</v>
@@ -64347,7 +64423,7 @@
       <c r="Y110" s="185"/>
       <c r="Z110" s="185"/>
       <c r="AA110" s="4" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="AB110" s="4">
         <v>-14.0</v>
@@ -64381,7 +64457,7 @@
       <c r="Y111" s="185"/>
       <c r="Z111" s="185"/>
       <c r="AA111" s="4" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="AB111" s="4">
         <v>-6.0</v>
@@ -64415,7 +64491,7 @@
       <c r="Y112" s="185"/>
       <c r="Z112" s="185"/>
       <c r="AA112" s="4" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="AB112" s="4">
         <v>-11.0</v>
@@ -64478,7 +64554,7 @@
       <c r="Y114" s="185"/>
       <c r="Z114" s="185"/>
       <c r="AA114" s="4" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="AB114" s="4">
         <v>-1.0</v>
@@ -64570,7 +64646,7 @@
       <c r="Y117" s="185"/>
       <c r="Z117" s="185"/>
       <c r="AA117" s="4" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="AB117" s="4">
         <v>12.0</v>
@@ -64633,7 +64709,7 @@
       <c r="Y119" s="185"/>
       <c r="Z119" s="185"/>
       <c r="AA119" s="4" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="AB119" s="4">
         <v>-17.0</v>
@@ -64754,7 +64830,7 @@
       <c r="Y123" s="185"/>
       <c r="Z123" s="185"/>
       <c r="AA123" s="4" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="AB123" s="4">
         <v>-15.0</v>
@@ -64905,7 +64981,7 @@
       <c r="Y128" s="185"/>
       <c r="Z128" s="185"/>
       <c r="AA128" s="4" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="AB128" s="4">
         <v>-11.0</v>
@@ -65290,7 +65366,7 @@
       <c r="Y141" s="185"/>
       <c r="Z141" s="185"/>
       <c r="AA141" s="4" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="AB141" s="4">
         <v>-10.0</v>

</xml_diff>